<commit_message>
Catalog: add mid-week Rosh Chodesh span note rule; enrich Elul customs rule
Rule 12i (new): the 'Rosh Chodesh: from X night to Y afternoon' note printed
in the zmanim block for mid-week Rosh Chodesh - the mining pass had excluded
RC notes as template, so a direct archive search recovered 15 instances with
varying wording (open question: canonical form). Rule 8a upgraded to two-year
evidence with the fuller 5786 Shoftim wording (LDavid from 1 Elul, shofar +
3 Tehillim daily from 2 Elul), supplied by the shul post-mining. Both review
spreadsheets regenerated (now 89 rules).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UeM1t6aqcLLPiTUiTN3paz
</commit_message>
<xml_diff>
--- a/phase0/mining/TTCC-special-days-review-SIMPLE.xlsx
+++ b/phase0/mining/TTCC-special-days-review-SIMPLE.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Timesheet rules'!$A$5:$H$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Timesheet rules'!$A$5:$H$94</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H93"/>
+  <dimension ref="A1:H94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2360,17 +2360,17 @@
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t>On Rosh Chodesh Elul.</t>
+          <t>The week containing Rosh Chodesh Elul.</t>
         </is>
       </c>
       <c r="D62" s="8" t="inlineStr">
         <is>
-          <t>Prints a note about starting L'David Hashem Ori at Shacharis and Mincha, practicing shofar blowing, and from 2 Elul, blowing shofar daily plus three extra chapters of Tehillim (for example, Monday = Tehillim 1-3, and so on).</t>
+          <t>Notes for the Elul customs, phrased by weekday: from 1 Elul, "add 'L'David Adn.. Ori' in Shacharis and Mincha"; from 2 Elul, "sound the shofar at the end of Shacharis (excl. Shabbos) and say three extra Tehillim", with the daily chapters spelled out (e.g. "On Fri. say Tehillim 1–3; on Shabbos say Tehillim 4–6 and so on").</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
-          <t>Standing Rosh Chodesh Elul custom note, seen once.</t>
+          <t>Shoftim 5786 (26 Av–2 Elul): "From Thurs. add 'L'David Adn.. Ori'… From Fri. sound the shofar… (On Fri. say Tehillim 1–3…)"</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr"/>
@@ -3339,10 +3339,44 @@
       <c r="G93" s="6" t="inlineStr"/>
       <c r="H93" s="6" t="inlineStr"/>
     </row>
+    <row r="94">
+      <c r="A94" s="7" t="inlineStr">
+        <is>
+          <t>12i</t>
+        </is>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>Calendar labels &amp; other notes</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="inlineStr">
+        <is>
+          <t>Any week where Rosh Chodesh falls on a weekday.</t>
+        </is>
+      </c>
+      <c r="D94" s="7" t="inlineStr">
+        <is>
+          <t>A note in the top block saying when Rosh Chodesh runs, starting from the evening before — for example "Rosh Chodesh: from Wed. night to Fri. afternoon." for a two-day Rosh Chodesh.</t>
+        </is>
+      </c>
+      <c r="E94" s="7" t="inlineStr">
+        <is>
+          <t>Shoftim 5786: "Rosh Chodesh: from Wed. night to Fri. afternoon." — 15 more examples found across past sheets, with slightly varying wording.</t>
+        </is>
+      </c>
+      <c r="F94" s="7" t="inlineStr">
+        <is>
+          <t>Past sheets vary the wording ("evening"/"night"/"afternoon", with or without the month's name). What should the standard wording be?</t>
+        </is>
+      </c>
+      <c r="G94" s="6" t="inlineStr"/>
+      <c r="H94" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:H93"/>
+  <autoFilter ref="A5:H94"/>
   <dataValidations count="1">
-    <dataValidation sqref="G6:G93" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G94" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Looks right,Needs a change (see notes),Leave it out,Not sure"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>